<commit_message>
Fix the Ebios RM matrix
</commit_message>
<xml_diff>
--- a/tools/matrix/risk-matrix-4x4-ebios-rm.xlsx
+++ b/tools/matrix/risk-matrix-4x4-ebios-rm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C7317E-59BF-0440-9A86-E157EDBFB29F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0B23ED-24F4-014E-90F8-93E13937D7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3860" yWindow="-28300" windowWidth="51200" windowHeight="28300" xr2:uid="{737B4EAE-987D-4047-A963-C4AA7BEFCFC2}"/>
+    <workbookView xWindow="3860" yWindow="-28300" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{737B4EAE-987D-4047-A963-C4AA7BEFCFC2}"/>
   </bookViews>
   <sheets>
     <sheet name="library_content" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="94">
   <si>
     <t>library_urn</t>
   </si>
@@ -162,24 +162,6 @@
     <t>Matrice 4x4 EBIOS-RM</t>
   </si>
   <si>
-    <t>G1 - Mineur</t>
-  </si>
-  <si>
-    <t>G1 - Minor</t>
-  </si>
-  <si>
-    <t>G2 - Significant</t>
-  </si>
-  <si>
-    <t>G2 - Significatif</t>
-  </si>
-  <si>
-    <t>G3 - Important</t>
-  </si>
-  <si>
-    <t>G4 - Critique</t>
-  </si>
-  <si>
     <t>Aucun impact opérationnel ni sur les performances de l’activité ni sur la sécurité des personnes et des biens.</t>
   </si>
   <si>
@@ -216,33 +198,12 @@
     <t>V4</t>
   </si>
   <si>
-    <t>V1 - Peu vraisemblable</t>
-  </si>
-  <si>
-    <t>V1 - Implausible</t>
-  </si>
-  <si>
-    <t>V2 - Plausible</t>
-  </si>
-  <si>
-    <t>V2 - Vraisemblable</t>
-  </si>
-  <si>
     <t>La source de risque a peu de chances d’atteindre son objectif visé selon l’un des modes opératoires envisagés. La vraisemblance du scénario est faible.</t>
   </si>
   <si>
     <t>La source de risque est susceptible d’atteindre son objectif visé selon l’un des modes opératoires envisagés. La vraisemblance du scénario est significative.</t>
   </si>
   <si>
-    <t>V3 - Très vraisemblable</t>
-  </si>
-  <si>
-    <t>V3 - Very likely</t>
-  </si>
-  <si>
-    <t>V4 - Certain</t>
-  </si>
-  <si>
     <t>La source de risque va probablement atteindre son objectif visé selon l’un des modes opératoires envisagés. La vraisemblance du scénario est élevée.</t>
   </si>
   <si>
@@ -316,6 +277,48 @@
   </si>
   <si>
     <t>urn:intuitem:risk:matrix:risk-matrix-4x4-ebios-rm</t>
+  </si>
+  <si>
+    <t>Certain</t>
+  </si>
+  <si>
+    <t>Très vraisemblable</t>
+  </si>
+  <si>
+    <t>Vraisemblable</t>
+  </si>
+  <si>
+    <t>Peu vraisemblable</t>
+  </si>
+  <si>
+    <t>Mineur</t>
+  </si>
+  <si>
+    <t>Significatif</t>
+  </si>
+  <si>
+    <t>Important</t>
+  </si>
+  <si>
+    <t>Critique</t>
+  </si>
+  <si>
+    <t>Very likely</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>Significant</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Likely</t>
+  </si>
+  <si>
+    <t>Unlikely</t>
   </si>
 </sst>
 </file>
@@ -892,7 +895,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -924,7 +927,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -956,7 +959,7 @@
         <v>20</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -980,7 +983,7 @@
         <v>23</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -1007,12 +1010,12 @@
         <v>32</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>40</v>
@@ -1023,7 +1026,7 @@
         <v>33</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1094,13 +1097,13 @@
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="G2" s="14">
         <v>1</v>
@@ -1115,10 +1118,10 @@
         <v>2</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1130,13 +1133,13 @@
       </c>
       <c r="C3" s="18"/>
       <c r="D3" s="6" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="G3" s="15">
         <v>0</v>
@@ -1151,10 +1154,10 @@
         <v>2</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1166,13 +1169,13 @@
       </c>
       <c r="C4" s="19"/>
       <c r="D4" s="6" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="G4" s="15">
         <v>0</v>
@@ -1187,10 +1190,10 @@
         <v>2</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1202,13 +1205,13 @@
       </c>
       <c r="C5" s="20"/>
       <c r="D5" s="6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="G5" s="15">
         <v>0</v>
@@ -1223,10 +1226,10 @@
         <v>1</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1238,19 +1241,19 @@
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="6" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="K6" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1262,19 +1265,19 @@
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="6" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>44</v>
+        <v>85</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1286,19 +1289,19 @@
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="6" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1310,19 +1313,19 @@
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="6" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>46</v>
+        <v>91</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.2">
@@ -1337,16 +1340,16 @@
         <v>28</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="51" x14ac:dyDescent="0.2">
@@ -1361,16 +1364,16 @@
         <v>29</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
@@ -1385,16 +1388,16 @@
         <v>30</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
fix(lib): EBIOS-RM matrix (#1935)
</commit_message>
<xml_diff>
--- a/tools/matrix/risk-matrix-4x4-ebios-rm.xlsx
+++ b/tools/matrix/risk-matrix-4x4-ebios-rm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/matrix/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE16766-2DDC-2A45-B2F6-C7A88AC9BDC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA767CD4-4D86-FF44-A17A-FD349432CBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20580" xr2:uid="{737B4EAE-987D-4047-A963-C4AA7BEFCFC2}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20260" xr2:uid="{737B4EAE-987D-4047-A963-C4AA7BEFCFC2}"/>
   </bookViews>
   <sheets>
     <sheet name="library_content" sheetId="1" r:id="rId1"/>
@@ -898,7 +898,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1111,8 +1111,8 @@
       <c r="G2" s="14">
         <v>1</v>
       </c>
-      <c r="H2" s="14">
-        <v>1</v>
+      <c r="H2" s="13">
+        <v>2</v>
       </c>
       <c r="I2" s="13">
         <v>2</v>
@@ -1144,8 +1144,8 @@
       <c r="F3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G3" s="15">
-        <v>0</v>
+      <c r="G3" s="14">
+        <v>1</v>
       </c>
       <c r="H3" s="14">
         <v>1</v>
@@ -1189,8 +1189,8 @@
       <c r="I4" s="14">
         <v>1</v>
       </c>
-      <c r="J4" s="13">
-        <v>2</v>
+      <c r="J4" s="14">
+        <v>1</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>82</v>
@@ -1222,8 +1222,8 @@
       <c r="H5" s="15">
         <v>0</v>
       </c>
-      <c r="I5" s="14">
-        <v>1</v>
+      <c r="I5" s="15">
+        <v>0</v>
       </c>
       <c r="J5" s="14">
         <v>1</v>

</xml_diff>